<commit_message>
Fix 500 error API by upgrading Gemini model and restrict bot suggestions to latest 2 properties
</commit_message>
<xml_diff>
--- a/Leased properties dataset Updated.xlsx
+++ b/Leased properties dataset Updated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bhims\.gemini\antigravity\scratch\qterra-chatbot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{00F459FD-6115-464B-9682-42A10B0910B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CF3955A-8438-42C0-9DAC-629F98998362}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{08F1B4CF-DD47-45C9-BC8B-73DCE3BF48B1}"/>
   </bookViews>
@@ -755,7 +755,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>

</xml_diff>